<commit_message>
feat: add admin ability to reset all student submissions
</commit_message>
<xml_diff>
--- a/Data_Akun_SkillPassport.xlsx
+++ b/Data_Akun_SkillPassport.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Private\Website\skillpas-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{384F14FD-6897-4224-9BB6-417AD2D7BECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE09A76-833F-41B0-A4E1-49D27AABD72E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Akun Staff" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="301">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -917,6 +930,12 @@
   </si>
   <si>
     <t>walas_yusuf_x_anim1_02</t>
+  </si>
+  <si>
+    <t>Guru Produktif Mesin 02</t>
+  </si>
+  <si>
+    <t>prod_mesin_02</t>
   </si>
 </sst>
 </file>
@@ -952,8 +971,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1293,8 +1315,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D160"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D161"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.796875" customWidth="1"/>
     <col min="2" max="2" width="20.796875" customWidth="1"/>
@@ -1304,7 +1326,7 @@
     <col min="6" max="7" width="36.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1318,7 +1340,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1332,7 +1354,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1346,7 +1368,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1360,7 +1382,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1374,7 +1396,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1388,7 +1410,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1402,7 +1424,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1416,7 +1438,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1430,7 +1452,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1444,7 +1466,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1458,7 +1480,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1472,7 +1494,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -1486,7 +1508,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1500,7 +1522,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -1514,7 +1536,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -1528,7 +1550,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -1542,7 +1564,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -1556,7 +1578,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -1570,7 +1592,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -1584,7 +1606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -1598,7 +1620,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -1612,7 +1634,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -1626,7 +1648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>53</v>
       </c>
@@ -1640,175 +1662,175 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>299</v>
       </c>
       <c r="B25" t="s">
         <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>300</v>
+      </c>
+      <c r="D25" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B26" t="s">
         <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s">
         <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D27" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s">
         <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D28" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s">
         <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B30" t="s">
         <v>45</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B31" t="s">
         <v>45</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32" t="s">
         <v>45</v>
       </c>
       <c r="C32" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" t="s">
         <v>70</v>
       </c>
-      <c r="D32" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
         <v>71</v>
       </c>
-      <c r="B33" t="s">
-        <v>72</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" t="s">
         <v>73</v>
       </c>
-      <c r="D33" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>74</v>
       </c>
-      <c r="B34" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="B35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" t="s">
         <v>75</v>
       </c>
-      <c r="D34" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>76</v>
       </c>
-      <c r="B35" t="s">
-        <v>72</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" t="s">
         <v>77</v>
       </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" t="s">
-        <v>72</v>
-      </c>
-      <c r="C36" t="s">
-        <v>79</v>
-      </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>78</v>
       </c>
@@ -1816,111 +1838,111 @@
         <v>72</v>
       </c>
       <c r="C37" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" t="s">
         <v>80</v>
       </c>
-      <c r="D37" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>81</v>
       </c>
-      <c r="B38" t="s">
-        <v>72</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="B39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" t="s">
         <v>82</v>
       </c>
-      <c r="D38" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>83</v>
       </c>
-      <c r="B39" t="s">
-        <v>72</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="B40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" t="s">
         <v>84</v>
       </c>
-      <c r="D39" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>85</v>
       </c>
-      <c r="B40" t="s">
-        <v>72</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="B41" t="s">
+        <v>72</v>
+      </c>
+      <c r="C41" t="s">
         <v>86</v>
       </c>
-      <c r="D40" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>87</v>
       </c>
-      <c r="B41" t="s">
-        <v>72</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="B42" t="s">
+        <v>72</v>
+      </c>
+      <c r="C42" t="s">
         <v>88</v>
       </c>
-      <c r="D41" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>89</v>
       </c>
-      <c r="B42" t="s">
-        <v>72</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="B43" t="s">
+        <v>72</v>
+      </c>
+      <c r="C43" t="s">
         <v>90</v>
       </c>
-      <c r="D42" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>91</v>
       </c>
-      <c r="B43" t="s">
-        <v>72</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B44" t="s">
+        <v>72</v>
+      </c>
+      <c r="C44" t="s">
         <v>92</v>
       </c>
-      <c r="D43" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>93</v>
-      </c>
-      <c r="B44" t="s">
-        <v>72</v>
-      </c>
-      <c r="C44" t="s">
-        <v>94</v>
-      </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>93</v>
       </c>
@@ -1928,69 +1950,69 @@
         <v>72</v>
       </c>
       <c r="C45" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>93</v>
+      </c>
+      <c r="B46" t="s">
+        <v>72</v>
+      </c>
+      <c r="C46" t="s">
         <v>95</v>
       </c>
-      <c r="D45" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>96</v>
       </c>
-      <c r="B46" t="s">
-        <v>72</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="B47" t="s">
+        <v>72</v>
+      </c>
+      <c r="C47" t="s">
         <v>97</v>
       </c>
-      <c r="D46" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
         <v>98</v>
       </c>
-      <c r="B47" t="s">
-        <v>72</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="B48" t="s">
+        <v>72</v>
+      </c>
+      <c r="C48" t="s">
         <v>99</v>
       </c>
-      <c r="D47" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
+      <c r="D48" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>100</v>
       </c>
-      <c r="B48" t="s">
-        <v>72</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="B49" t="s">
+        <v>72</v>
+      </c>
+      <c r="C49" t="s">
         <v>101</v>
       </c>
-      <c r="D48" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>102</v>
-      </c>
-      <c r="B49" t="s">
-        <v>72</v>
-      </c>
-      <c r="C49" t="s">
-        <v>103</v>
-      </c>
       <c r="D49" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>102</v>
       </c>
@@ -1998,69 +2020,69 @@
         <v>72</v>
       </c>
       <c r="C50" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" t="s">
+        <v>72</v>
+      </c>
+      <c r="C51" t="s">
         <v>104</v>
       </c>
-      <c r="D50" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
         <v>18</v>
       </c>
-      <c r="B51" t="s">
-        <v>72</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="B52" t="s">
+        <v>72</v>
+      </c>
+      <c r="C52" t="s">
         <v>105</v>
       </c>
-      <c r="D51" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>106</v>
       </c>
-      <c r="B52" t="s">
-        <v>72</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="B53" t="s">
+        <v>72</v>
+      </c>
+      <c r="C53" t="s">
         <v>107</v>
       </c>
-      <c r="D52" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>108</v>
       </c>
-      <c r="B53" t="s">
-        <v>72</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="B54" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" t="s">
         <v>109</v>
       </c>
-      <c r="D53" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>110</v>
-      </c>
-      <c r="B54" t="s">
-        <v>72</v>
-      </c>
-      <c r="C54" t="s">
-        <v>111</v>
-      </c>
       <c r="D54" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>110</v>
       </c>
@@ -2068,27 +2090,27 @@
         <v>72</v>
       </c>
       <c r="C55" t="s">
+        <v>111</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" t="s">
+        <v>72</v>
+      </c>
+      <c r="C56" t="s">
         <v>112</v>
       </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>113</v>
-      </c>
-      <c r="B56" t="s">
-        <v>72</v>
-      </c>
-      <c r="C56" t="s">
-        <v>114</v>
-      </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>113</v>
       </c>
@@ -2096,125 +2118,125 @@
         <v>72</v>
       </c>
       <c r="C57" t="s">
+        <v>114</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58" t="s">
         <v>115</v>
       </c>
-      <c r="D57" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>116</v>
       </c>
-      <c r="B58" t="s">
-        <v>72</v>
-      </c>
-      <c r="C58" t="s">
+      <c r="B59" t="s">
+        <v>72</v>
+      </c>
+      <c r="C59" t="s">
         <v>117</v>
       </c>
-      <c r="D58" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>118</v>
       </c>
-      <c r="B59" t="s">
-        <v>72</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="B60" t="s">
+        <v>72</v>
+      </c>
+      <c r="C60" t="s">
         <v>119</v>
       </c>
-      <c r="D59" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>120</v>
       </c>
-      <c r="B60" t="s">
-        <v>72</v>
-      </c>
-      <c r="C60" t="s">
+      <c r="B61" t="s">
+        <v>72</v>
+      </c>
+      <c r="C61" t="s">
         <v>121</v>
       </c>
-      <c r="D60" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
         <v>122</v>
       </c>
-      <c r="B61" t="s">
-        <v>72</v>
-      </c>
-      <c r="C61" t="s">
+      <c r="B62" t="s">
+        <v>72</v>
+      </c>
+      <c r="C62" t="s">
         <v>123</v>
       </c>
-      <c r="D61" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>124</v>
       </c>
-      <c r="B62" t="s">
-        <v>72</v>
-      </c>
-      <c r="C62" t="s">
+      <c r="B63" t="s">
+        <v>72</v>
+      </c>
+      <c r="C63" t="s">
         <v>125</v>
       </c>
-      <c r="D62" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
         <v>126</v>
       </c>
-      <c r="B63" t="s">
-        <v>72</v>
-      </c>
-      <c r="C63" t="s">
+      <c r="B64" t="s">
+        <v>72</v>
+      </c>
+      <c r="C64" t="s">
         <v>127</v>
       </c>
-      <c r="D63" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
+      <c r="D64" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
         <v>128</v>
       </c>
-      <c r="B64" t="s">
-        <v>72</v>
-      </c>
-      <c r="C64" t="s">
+      <c r="B65" t="s">
+        <v>72</v>
+      </c>
+      <c r="C65" t="s">
         <v>129</v>
       </c>
-      <c r="D64" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>130</v>
-      </c>
-      <c r="B65" t="s">
-        <v>72</v>
-      </c>
-      <c r="C65" t="s">
-        <v>131</v>
-      </c>
       <c r="D65" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>130</v>
       </c>
@@ -2222,69 +2244,69 @@
         <v>72</v>
       </c>
       <c r="C66" t="s">
+        <v>131</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" t="s">
+        <v>72</v>
+      </c>
+      <c r="C67" t="s">
         <v>132</v>
       </c>
-      <c r="D66" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
         <v>133</v>
       </c>
-      <c r="B67" t="s">
-        <v>72</v>
-      </c>
-      <c r="C67" t="s">
+      <c r="B68" t="s">
+        <v>72</v>
+      </c>
+      <c r="C68" t="s">
         <v>134</v>
       </c>
-      <c r="D67" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>135</v>
       </c>
-      <c r="B68" t="s">
-        <v>72</v>
-      </c>
-      <c r="C68" t="s">
+      <c r="B69" t="s">
+        <v>72</v>
+      </c>
+      <c r="C69" t="s">
         <v>136</v>
       </c>
-      <c r="D68" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>137</v>
       </c>
-      <c r="B69" t="s">
-        <v>72</v>
-      </c>
-      <c r="C69" t="s">
+      <c r="B70" t="s">
+        <v>72</v>
+      </c>
+      <c r="C70" t="s">
         <v>138</v>
       </c>
-      <c r="D69" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>139</v>
-      </c>
-      <c r="B70" t="s">
-        <v>72</v>
-      </c>
-      <c r="C70" t="s">
-        <v>140</v>
-      </c>
       <c r="D70" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>139</v>
       </c>
@@ -2292,27 +2314,27 @@
         <v>72</v>
       </c>
       <c r="C71" t="s">
+        <v>140</v>
+      </c>
+      <c r="D71" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>139</v>
+      </c>
+      <c r="B72" t="s">
+        <v>72</v>
+      </c>
+      <c r="C72" t="s">
         <v>141</v>
       </c>
-      <c r="D71" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>142</v>
-      </c>
-      <c r="B72" t="s">
-        <v>72</v>
-      </c>
-      <c r="C72" t="s">
-        <v>143</v>
-      </c>
       <c r="D72" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>142</v>
       </c>
@@ -2320,69 +2342,69 @@
         <v>72</v>
       </c>
       <c r="C73" t="s">
+        <v>143</v>
+      </c>
+      <c r="D73" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>142</v>
+      </c>
+      <c r="B74" t="s">
+        <v>72</v>
+      </c>
+      <c r="C74" t="s">
         <v>144</v>
       </c>
-      <c r="D73" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
+      <c r="D74" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
         <v>20</v>
       </c>
-      <c r="B74" t="s">
-        <v>72</v>
-      </c>
-      <c r="C74" t="s">
+      <c r="B75" t="s">
+        <v>72</v>
+      </c>
+      <c r="C75" t="s">
         <v>145</v>
       </c>
-      <c r="D74" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
+      <c r="D75" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
         <v>146</v>
       </c>
-      <c r="B75" t="s">
-        <v>72</v>
-      </c>
-      <c r="C75" t="s">
+      <c r="B76" t="s">
+        <v>72</v>
+      </c>
+      <c r="C76" t="s">
         <v>147</v>
       </c>
-      <c r="D75" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
+      <c r="D76" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
         <v>148</v>
       </c>
-      <c r="B76" t="s">
-        <v>72</v>
-      </c>
-      <c r="C76" t="s">
+      <c r="B77" t="s">
+        <v>72</v>
+      </c>
+      <c r="C77" t="s">
         <v>149</v>
       </c>
-      <c r="D76" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>150</v>
-      </c>
-      <c r="B77" t="s">
-        <v>72</v>
-      </c>
-      <c r="C77" t="s">
-        <v>151</v>
-      </c>
       <c r="D77" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>150</v>
       </c>
@@ -2390,27 +2412,27 @@
         <v>72</v>
       </c>
       <c r="C78" t="s">
+        <v>151</v>
+      </c>
+      <c r="D78" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>150</v>
+      </c>
+      <c r="B79" t="s">
+        <v>72</v>
+      </c>
+      <c r="C79" t="s">
         <v>152</v>
       </c>
-      <c r="D78" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>153</v>
-      </c>
-      <c r="B79" t="s">
-        <v>72</v>
-      </c>
-      <c r="C79" t="s">
-        <v>154</v>
-      </c>
       <c r="D79" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>153</v>
       </c>
@@ -2418,83 +2440,83 @@
         <v>72</v>
       </c>
       <c r="C80" t="s">
+        <v>154</v>
+      </c>
+      <c r="D80" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>153</v>
+      </c>
+      <c r="B81" t="s">
+        <v>72</v>
+      </c>
+      <c r="C81" t="s">
         <v>155</v>
       </c>
-      <c r="D80" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
+      <c r="D81" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
         <v>156</v>
       </c>
-      <c r="B81" t="s">
-        <v>72</v>
-      </c>
-      <c r="C81" t="s">
+      <c r="B82" t="s">
+        <v>72</v>
+      </c>
+      <c r="C82" t="s">
         <v>157</v>
       </c>
-      <c r="D81" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
+      <c r="D82" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
         <v>158</v>
       </c>
-      <c r="B82" t="s">
-        <v>72</v>
-      </c>
-      <c r="C82" t="s">
+      <c r="B83" t="s">
+        <v>72</v>
+      </c>
+      <c r="C83" t="s">
         <v>159</v>
       </c>
-      <c r="D82" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
+      <c r="D83" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
         <v>160</v>
       </c>
-      <c r="B83" t="s">
-        <v>72</v>
-      </c>
-      <c r="C83" t="s">
+      <c r="B84" t="s">
+        <v>72</v>
+      </c>
+      <c r="C84" t="s">
         <v>161</v>
       </c>
-      <c r="D83" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
+      <c r="D84" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
         <v>162</v>
       </c>
-      <c r="B84" t="s">
-        <v>72</v>
-      </c>
-      <c r="C84" t="s">
+      <c r="B85" t="s">
+        <v>72</v>
+      </c>
+      <c r="C85" t="s">
         <v>163</v>
       </c>
-      <c r="D84" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>164</v>
-      </c>
-      <c r="B85" t="s">
-        <v>72</v>
-      </c>
-      <c r="C85" t="s">
-        <v>165</v>
-      </c>
       <c r="D85" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>164</v>
       </c>
@@ -2502,55 +2524,55 @@
         <v>72</v>
       </c>
       <c r="C86" t="s">
+        <v>165</v>
+      </c>
+      <c r="D86" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>164</v>
+      </c>
+      <c r="B87" t="s">
+        <v>72</v>
+      </c>
+      <c r="C87" t="s">
         <v>166</v>
       </c>
-      <c r="D86" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
+      <c r="D87" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
         <v>167</v>
       </c>
-      <c r="B87" t="s">
-        <v>72</v>
-      </c>
-      <c r="C87" t="s">
+      <c r="B88" t="s">
+        <v>72</v>
+      </c>
+      <c r="C88" t="s">
         <v>168</v>
       </c>
-      <c r="D87" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
+      <c r="D88" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
         <v>169</v>
       </c>
-      <c r="B88" t="s">
-        <v>72</v>
-      </c>
-      <c r="C88" t="s">
+      <c r="B89" t="s">
+        <v>72</v>
+      </c>
+      <c r="C89" t="s">
         <v>170</v>
       </c>
-      <c r="D88" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>171</v>
-      </c>
-      <c r="B89" t="s">
-        <v>72</v>
-      </c>
-      <c r="C89" t="s">
-        <v>172</v>
-      </c>
       <c r="D89" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>171</v>
       </c>
@@ -2558,27 +2580,27 @@
         <v>72</v>
       </c>
       <c r="C90" t="s">
+        <v>172</v>
+      </c>
+      <c r="D90" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>171</v>
+      </c>
+      <c r="B91" t="s">
+        <v>72</v>
+      </c>
+      <c r="C91" t="s">
         <v>173</v>
       </c>
-      <c r="D90" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>174</v>
-      </c>
-      <c r="B91" t="s">
-        <v>72</v>
-      </c>
-      <c r="C91" t="s">
-        <v>175</v>
-      </c>
       <c r="D91" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>174</v>
       </c>
@@ -2586,27 +2608,27 @@
         <v>72</v>
       </c>
       <c r="C92" t="s">
+        <v>175</v>
+      </c>
+      <c r="D92" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>174</v>
+      </c>
+      <c r="B93" t="s">
+        <v>72</v>
+      </c>
+      <c r="C93" t="s">
         <v>176</v>
       </c>
-      <c r="D92" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>177</v>
-      </c>
-      <c r="B93" t="s">
-        <v>72</v>
-      </c>
-      <c r="C93" t="s">
-        <v>178</v>
-      </c>
       <c r="D93" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>177</v>
       </c>
@@ -2614,97 +2636,97 @@
         <v>72</v>
       </c>
       <c r="C94" t="s">
+        <v>178</v>
+      </c>
+      <c r="D94" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>177</v>
+      </c>
+      <c r="B95" t="s">
+        <v>72</v>
+      </c>
+      <c r="C95" t="s">
         <v>179</v>
       </c>
-      <c r="D94" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
+      <c r="D95" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
         <v>180</v>
       </c>
-      <c r="B95" t="s">
-        <v>72</v>
-      </c>
-      <c r="C95" t="s">
+      <c r="B96" t="s">
+        <v>72</v>
+      </c>
+      <c r="C96" t="s">
         <v>181</v>
       </c>
-      <c r="D95" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+      <c r="D96" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>182</v>
       </c>
-      <c r="B96" t="s">
-        <v>72</v>
-      </c>
-      <c r="C96" t="s">
+      <c r="B97" t="s">
+        <v>72</v>
+      </c>
+      <c r="C97" t="s">
         <v>183</v>
       </c>
-      <c r="D96" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
+      <c r="D97" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
         <v>184</v>
       </c>
-      <c r="B97" t="s">
-        <v>72</v>
-      </c>
-      <c r="C97" t="s">
+      <c r="B98" t="s">
+        <v>72</v>
+      </c>
+      <c r="C98" t="s">
         <v>185</v>
       </c>
-      <c r="D97" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
+      <c r="D98" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
         <v>186</v>
       </c>
-      <c r="B98" t="s">
-        <v>72</v>
-      </c>
-      <c r="C98" t="s">
+      <c r="B99" t="s">
+        <v>72</v>
+      </c>
+      <c r="C99" t="s">
         <v>187</v>
       </c>
-      <c r="D98" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
+      <c r="D99" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
         <v>188</v>
       </c>
-      <c r="B99" t="s">
-        <v>72</v>
-      </c>
-      <c r="C99" t="s">
+      <c r="B100" t="s">
+        <v>72</v>
+      </c>
+      <c r="C100" t="s">
         <v>189</v>
       </c>
-      <c r="D99" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
-        <v>190</v>
-      </c>
-      <c r="B100" t="s">
-        <v>72</v>
-      </c>
-      <c r="C100" t="s">
-        <v>191</v>
-      </c>
       <c r="D100" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>190</v>
       </c>
@@ -2712,27 +2734,27 @@
         <v>72</v>
       </c>
       <c r="C101" t="s">
+        <v>191</v>
+      </c>
+      <c r="D101" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>190</v>
+      </c>
+      <c r="B102" t="s">
+        <v>72</v>
+      </c>
+      <c r="C102" t="s">
         <v>192</v>
       </c>
-      <c r="D101" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
-        <v>193</v>
-      </c>
-      <c r="B102" t="s">
-        <v>72</v>
-      </c>
-      <c r="C102" t="s">
-        <v>194</v>
-      </c>
       <c r="D102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>193</v>
       </c>
@@ -2740,41 +2762,41 @@
         <v>72</v>
       </c>
       <c r="C103" t="s">
+        <v>194</v>
+      </c>
+      <c r="D103" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" t="s">
+        <v>72</v>
+      </c>
+      <c r="C104" t="s">
         <v>195</v>
       </c>
-      <c r="D103" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
+      <c r="D104" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
         <v>196</v>
       </c>
-      <c r="B104" t="s">
-        <v>72</v>
-      </c>
-      <c r="C104" t="s">
+      <c r="B105" t="s">
+        <v>72</v>
+      </c>
+      <c r="C105" t="s">
         <v>197</v>
       </c>
-      <c r="D104" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>198</v>
-      </c>
-      <c r="B105" t="s">
-        <v>72</v>
-      </c>
-      <c r="C105" t="s">
-        <v>199</v>
-      </c>
       <c r="D105" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>198</v>
       </c>
@@ -2782,69 +2804,69 @@
         <v>72</v>
       </c>
       <c r="C106" t="s">
+        <v>199</v>
+      </c>
+      <c r="D106" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>198</v>
+      </c>
+      <c r="B107" t="s">
+        <v>72</v>
+      </c>
+      <c r="C107" t="s">
         <v>200</v>
       </c>
-      <c r="D106" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
+      <c r="D107" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
         <v>201</v>
       </c>
-      <c r="B107" t="s">
-        <v>72</v>
-      </c>
-      <c r="C107" t="s">
+      <c r="B108" t="s">
+        <v>72</v>
+      </c>
+      <c r="C108" t="s">
         <v>202</v>
       </c>
-      <c r="D107" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
+      <c r="D108" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
         <v>203</v>
       </c>
-      <c r="B108" t="s">
-        <v>72</v>
-      </c>
-      <c r="C108" t="s">
+      <c r="B109" t="s">
+        <v>72</v>
+      </c>
+      <c r="C109" t="s">
         <v>204</v>
       </c>
-      <c r="D108" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
+      <c r="D109" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
         <v>205</v>
       </c>
-      <c r="B109" t="s">
-        <v>72</v>
-      </c>
-      <c r="C109" t="s">
+      <c r="B110" t="s">
+        <v>72</v>
+      </c>
+      <c r="C110" t="s">
         <v>206</v>
       </c>
-      <c r="D109" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A110" t="s">
-        <v>207</v>
-      </c>
-      <c r="B110" t="s">
-        <v>72</v>
-      </c>
-      <c r="C110" t="s">
-        <v>208</v>
-      </c>
       <c r="D110" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>207</v>
       </c>
@@ -2852,251 +2874,251 @@
         <v>72</v>
       </c>
       <c r="C111" t="s">
+        <v>208</v>
+      </c>
+      <c r="D111" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>207</v>
+      </c>
+      <c r="B112" t="s">
+        <v>72</v>
+      </c>
+      <c r="C112" t="s">
         <v>209</v>
       </c>
-      <c r="D111" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A112" t="s">
+      <c r="D112" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
         <v>210</v>
       </c>
-      <c r="B112" t="s">
-        <v>72</v>
-      </c>
-      <c r="C112" t="s">
+      <c r="B113" t="s">
+        <v>72</v>
+      </c>
+      <c r="C113" t="s">
         <v>211</v>
       </c>
-      <c r="D112" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
+      <c r="D113" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
         <v>212</v>
       </c>
-      <c r="B113" t="s">
-        <v>72</v>
-      </c>
-      <c r="C113" t="s">
+      <c r="B114" t="s">
+        <v>72</v>
+      </c>
+      <c r="C114" t="s">
         <v>213</v>
       </c>
-      <c r="D113" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A114" t="s">
+      <c r="D114" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
         <v>214</v>
       </c>
-      <c r="B114" t="s">
-        <v>72</v>
-      </c>
-      <c r="C114" t="s">
+      <c r="B115" t="s">
+        <v>72</v>
+      </c>
+      <c r="C115" t="s">
         <v>215</v>
       </c>
-      <c r="D114" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A115" t="s">
+      <c r="D115" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
         <v>216</v>
       </c>
-      <c r="B115" t="s">
-        <v>72</v>
-      </c>
-      <c r="C115" t="s">
+      <c r="B116" t="s">
+        <v>72</v>
+      </c>
+      <c r="C116" t="s">
         <v>217</v>
       </c>
-      <c r="D115" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
+      <c r="D116" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
         <v>218</v>
       </c>
-      <c r="B116" t="s">
-        <v>72</v>
-      </c>
-      <c r="C116" t="s">
+      <c r="B117" t="s">
+        <v>72</v>
+      </c>
+      <c r="C117" t="s">
         <v>219</v>
       </c>
-      <c r="D116" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
+      <c r="D117" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
         <v>220</v>
       </c>
-      <c r="B117" t="s">
-        <v>72</v>
-      </c>
-      <c r="C117" t="s">
+      <c r="B118" t="s">
+        <v>72</v>
+      </c>
+      <c r="C118" t="s">
         <v>221</v>
       </c>
-      <c r="D117" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
+      <c r="D118" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
         <v>222</v>
       </c>
-      <c r="B118" t="s">
-        <v>72</v>
-      </c>
-      <c r="C118" t="s">
+      <c r="B119" t="s">
+        <v>72</v>
+      </c>
+      <c r="C119" t="s">
         <v>223</v>
       </c>
-      <c r="D118" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
+      <c r="D119" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
         <v>224</v>
       </c>
-      <c r="B119" t="s">
-        <v>72</v>
-      </c>
-      <c r="C119" t="s">
+      <c r="B120" t="s">
+        <v>72</v>
+      </c>
+      <c r="C120" t="s">
         <v>225</v>
       </c>
-      <c r="D119" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
+      <c r="D120" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
         <v>226</v>
       </c>
-      <c r="B120" t="s">
-        <v>72</v>
-      </c>
-      <c r="C120" t="s">
+      <c r="B121" t="s">
+        <v>72</v>
+      </c>
+      <c r="C121" t="s">
         <v>227</v>
       </c>
-      <c r="D120" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A121" t="s">
+      <c r="D121" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
         <v>228</v>
       </c>
-      <c r="B121" t="s">
-        <v>72</v>
-      </c>
-      <c r="C121" t="s">
+      <c r="B122" t="s">
+        <v>72</v>
+      </c>
+      <c r="C122" t="s">
         <v>229</v>
       </c>
-      <c r="D121" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A122" t="s">
+      <c r="D122" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
         <v>230</v>
       </c>
-      <c r="B122" t="s">
-        <v>72</v>
-      </c>
-      <c r="C122" t="s">
+      <c r="B123" t="s">
+        <v>72</v>
+      </c>
+      <c r="C123" t="s">
         <v>231</v>
       </c>
-      <c r="D122" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A123" t="s">
+      <c r="D123" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
         <v>232</v>
       </c>
-      <c r="B123" t="s">
-        <v>72</v>
-      </c>
-      <c r="C123" t="s">
+      <c r="B124" t="s">
+        <v>72</v>
+      </c>
+      <c r="C124" t="s">
         <v>233</v>
       </c>
-      <c r="D123" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A124" t="s">
+      <c r="D124" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
         <v>234</v>
       </c>
-      <c r="B124" t="s">
-        <v>72</v>
-      </c>
-      <c r="C124" t="s">
+      <c r="B125" t="s">
+        <v>72</v>
+      </c>
+      <c r="C125" t="s">
         <v>235</v>
       </c>
-      <c r="D124" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A125" t="s">
+      <c r="D125" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
         <v>34</v>
       </c>
-      <c r="B125" t="s">
-        <v>72</v>
-      </c>
-      <c r="C125" t="s">
+      <c r="B126" t="s">
+        <v>72</v>
+      </c>
+      <c r="C126" t="s">
         <v>236</v>
       </c>
-      <c r="D125" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
+      <c r="D126" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
         <v>237</v>
       </c>
-      <c r="B126" t="s">
-        <v>72</v>
-      </c>
-      <c r="C126" t="s">
+      <c r="B127" t="s">
+        <v>72</v>
+      </c>
+      <c r="C127" t="s">
         <v>238</v>
       </c>
-      <c r="D126" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
+      <c r="D127" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
         <v>239</v>
       </c>
-      <c r="B127" t="s">
-        <v>72</v>
-      </c>
-      <c r="C127" t="s">
+      <c r="B128" t="s">
+        <v>72</v>
+      </c>
+      <c r="C128" t="s">
         <v>240</v>
       </c>
-      <c r="D127" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A128" t="s">
-        <v>241</v>
-      </c>
-      <c r="B128" t="s">
-        <v>72</v>
-      </c>
-      <c r="C128" t="s">
-        <v>242</v>
-      </c>
       <c r="D128" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>241</v>
       </c>
@@ -3104,55 +3126,55 @@
         <v>72</v>
       </c>
       <c r="C129" t="s">
+        <v>242</v>
+      </c>
+      <c r="D129" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>241</v>
+      </c>
+      <c r="B130" t="s">
+        <v>72</v>
+      </c>
+      <c r="C130" t="s">
         <v>243</v>
       </c>
-      <c r="D129" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
+      <c r="D130" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
         <v>244</v>
       </c>
-      <c r="B130" t="s">
-        <v>72</v>
-      </c>
-      <c r="C130" t="s">
+      <c r="B131" t="s">
+        <v>72</v>
+      </c>
+      <c r="C131" t="s">
         <v>245</v>
       </c>
-      <c r="D130" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A131" t="s">
+      <c r="D131" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
         <v>246</v>
       </c>
-      <c r="B131" t="s">
-        <v>72</v>
-      </c>
-      <c r="C131" t="s">
+      <c r="B132" t="s">
+        <v>72</v>
+      </c>
+      <c r="C132" t="s">
         <v>247</v>
       </c>
-      <c r="D131" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A132" t="s">
-        <v>248</v>
-      </c>
-      <c r="B132" t="s">
-        <v>72</v>
-      </c>
-      <c r="C132" t="s">
-        <v>249</v>
-      </c>
       <c r="D132" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>248</v>
       </c>
@@ -3160,55 +3182,55 @@
         <v>72</v>
       </c>
       <c r="C133" t="s">
+        <v>249</v>
+      </c>
+      <c r="D133" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>248</v>
+      </c>
+      <c r="B134" t="s">
+        <v>72</v>
+      </c>
+      <c r="C134" t="s">
         <v>250</v>
       </c>
-      <c r="D133" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A134" t="s">
+      <c r="D134" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
         <v>251</v>
       </c>
-      <c r="B134" t="s">
-        <v>72</v>
-      </c>
-      <c r="C134" t="s">
+      <c r="B135" t="s">
+        <v>72</v>
+      </c>
+      <c r="C135" t="s">
         <v>252</v>
       </c>
-      <c r="D134" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A135" t="s">
+      <c r="D135" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
         <v>253</v>
       </c>
-      <c r="B135" t="s">
-        <v>72</v>
-      </c>
-      <c r="C135" t="s">
+      <c r="B136" t="s">
+        <v>72</v>
+      </c>
+      <c r="C136" t="s">
         <v>254</v>
       </c>
-      <c r="D135" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A136" t="s">
-        <v>255</v>
-      </c>
-      <c r="B136" t="s">
-        <v>72</v>
-      </c>
-      <c r="C136" t="s">
-        <v>256</v>
-      </c>
       <c r="D136" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>255</v>
       </c>
@@ -3216,69 +3238,69 @@
         <v>72</v>
       </c>
       <c r="C137" t="s">
+        <v>256</v>
+      </c>
+      <c r="D137" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>255</v>
+      </c>
+      <c r="B138" t="s">
+        <v>72</v>
+      </c>
+      <c r="C138" t="s">
         <v>257</v>
       </c>
-      <c r="D137" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A138" t="s">
+      <c r="D138" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
         <v>258</v>
       </c>
-      <c r="B138" t="s">
-        <v>72</v>
-      </c>
-      <c r="C138" t="s">
+      <c r="B139" t="s">
+        <v>72</v>
+      </c>
+      <c r="C139" t="s">
         <v>259</v>
       </c>
-      <c r="D138" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A139" t="s">
+      <c r="D139" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
         <v>260</v>
       </c>
-      <c r="B139" t="s">
-        <v>72</v>
-      </c>
-      <c r="C139" t="s">
+      <c r="B140" t="s">
+        <v>72</v>
+      </c>
+      <c r="C140" t="s">
         <v>261</v>
       </c>
-      <c r="D139" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
+      <c r="D140" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
         <v>262</v>
       </c>
-      <c r="B140" t="s">
-        <v>72</v>
-      </c>
-      <c r="C140" t="s">
+      <c r="B141" t="s">
+        <v>72</v>
+      </c>
+      <c r="C141" t="s">
         <v>263</v>
       </c>
-      <c r="D140" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A141" t="s">
-        <v>264</v>
-      </c>
-      <c r="B141" t="s">
-        <v>72</v>
-      </c>
-      <c r="C141" t="s">
-        <v>265</v>
-      </c>
       <c r="D141" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>264</v>
       </c>
@@ -3286,83 +3308,83 @@
         <v>72</v>
       </c>
       <c r="C142" t="s">
+        <v>265</v>
+      </c>
+      <c r="D142" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>264</v>
+      </c>
+      <c r="B143" t="s">
+        <v>72</v>
+      </c>
+      <c r="C143" t="s">
         <v>266</v>
       </c>
-      <c r="D142" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A143" t="s">
+      <c r="D143" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
         <v>267</v>
       </c>
-      <c r="B143" t="s">
-        <v>72</v>
-      </c>
-      <c r="C143" t="s">
+      <c r="B144" t="s">
+        <v>72</v>
+      </c>
+      <c r="C144" t="s">
         <v>268</v>
       </c>
-      <c r="D143" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A144" t="s">
+      <c r="D144" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
         <v>269</v>
       </c>
-      <c r="B144" t="s">
-        <v>72</v>
-      </c>
-      <c r="C144" t="s">
+      <c r="B145" t="s">
+        <v>72</v>
+      </c>
+      <c r="C145" t="s">
         <v>270</v>
       </c>
-      <c r="D144" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A145" t="s">
+      <c r="D145" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
         <v>271</v>
       </c>
-      <c r="B145" t="s">
-        <v>72</v>
-      </c>
-      <c r="C145" t="s">
+      <c r="B146" t="s">
+        <v>72</v>
+      </c>
+      <c r="C146" t="s">
         <v>272</v>
       </c>
-      <c r="D145" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A146" t="s">
+      <c r="D146" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
         <v>273</v>
       </c>
-      <c r="B146" t="s">
-        <v>72</v>
-      </c>
-      <c r="C146" t="s">
+      <c r="B147" t="s">
+        <v>72</v>
+      </c>
+      <c r="C147" t="s">
         <v>274</v>
       </c>
-      <c r="D146" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A147" t="s">
-        <v>275</v>
-      </c>
-      <c r="B147" t="s">
-        <v>72</v>
-      </c>
-      <c r="C147" t="s">
-        <v>276</v>
-      </c>
       <c r="D147" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>275</v>
       </c>
@@ -3370,41 +3392,41 @@
         <v>72</v>
       </c>
       <c r="C148" t="s">
+        <v>276</v>
+      </c>
+      <c r="D148" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>275</v>
+      </c>
+      <c r="B149" t="s">
+        <v>72</v>
+      </c>
+      <c r="C149" t="s">
         <v>277</v>
       </c>
-      <c r="D148" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A149" t="s">
+      <c r="D149" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
         <v>278</v>
       </c>
-      <c r="B149" t="s">
-        <v>72</v>
-      </c>
-      <c r="C149" t="s">
+      <c r="B150" t="s">
+        <v>72</v>
+      </c>
+      <c r="C150" t="s">
         <v>279</v>
       </c>
-      <c r="D149" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A150" t="s">
-        <v>280</v>
-      </c>
-      <c r="B150" t="s">
-        <v>72</v>
-      </c>
-      <c r="C150" t="s">
-        <v>281</v>
-      </c>
       <c r="D150" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>280</v>
       </c>
@@ -3412,41 +3434,41 @@
         <v>72</v>
       </c>
       <c r="C151" t="s">
+        <v>281</v>
+      </c>
+      <c r="D151" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>280</v>
+      </c>
+      <c r="B152" t="s">
+        <v>72</v>
+      </c>
+      <c r="C152" t="s">
         <v>282</v>
       </c>
-      <c r="D151" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A152" t="s">
+      <c r="D152" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
         <v>283</v>
       </c>
-      <c r="B152" t="s">
-        <v>72</v>
-      </c>
-      <c r="C152" t="s">
+      <c r="B153" t="s">
+        <v>72</v>
+      </c>
+      <c r="C153" t="s">
         <v>284</v>
       </c>
-      <c r="D152" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A153" t="s">
-        <v>285</v>
-      </c>
-      <c r="B153" t="s">
-        <v>72</v>
-      </c>
-      <c r="C153" t="s">
-        <v>286</v>
-      </c>
       <c r="D153" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="154" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>285</v>
       </c>
@@ -3454,41 +3476,41 @@
         <v>72</v>
       </c>
       <c r="C154" t="s">
+        <v>286</v>
+      </c>
+      <c r="D154" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>285</v>
+      </c>
+      <c r="B155" t="s">
+        <v>72</v>
+      </c>
+      <c r="C155" t="s">
         <v>287</v>
       </c>
-      <c r="D154" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A155" t="s">
+      <c r="D155" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
         <v>288</v>
       </c>
-      <c r="B155" t="s">
-        <v>72</v>
-      </c>
-      <c r="C155" t="s">
+      <c r="B156" t="s">
+        <v>72</v>
+      </c>
+      <c r="C156" t="s">
         <v>289</v>
       </c>
-      <c r="D155" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A156" t="s">
-        <v>290</v>
-      </c>
-      <c r="B156" t="s">
-        <v>72</v>
-      </c>
-      <c r="C156" t="s">
-        <v>291</v>
-      </c>
       <c r="D156" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>290</v>
       </c>
@@ -3496,58 +3518,73 @@
         <v>72</v>
       </c>
       <c r="C157" t="s">
+        <v>291</v>
+      </c>
+      <c r="D157" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>290</v>
+      </c>
+      <c r="B158" t="s">
+        <v>72</v>
+      </c>
+      <c r="C158" t="s">
         <v>292</v>
       </c>
-      <c r="D157" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A158" t="s">
+      <c r="D158" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
         <v>293</v>
       </c>
-      <c r="B158" t="s">
-        <v>72</v>
-      </c>
-      <c r="C158" t="s">
+      <c r="B159" t="s">
+        <v>72</v>
+      </c>
+      <c r="C159" t="s">
         <v>294</v>
       </c>
-      <c r="D158" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A159" t="s">
+      <c r="D159" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
         <v>295</v>
       </c>
-      <c r="B159" t="s">
-        <v>72</v>
-      </c>
-      <c r="C159" t="s">
+      <c r="B160" t="s">
+        <v>72</v>
+      </c>
+      <c r="C160" t="s">
         <v>296</v>
       </c>
-      <c r="D159" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A160" t="s">
+      <c r="D160" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
         <v>297</v>
       </c>
-      <c r="B160" t="s">
-        <v>72</v>
-      </c>
-      <c r="C160" t="s">
+      <c r="B161" t="s">
+        <v>72</v>
+      </c>
+      <c r="C161" t="s">
         <v>298</v>
       </c>
-      <c r="D160" t="s">
+      <c r="D161" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D160" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D17 A27:B27 A26:B26 D26 A29:D161 A28:B28 D28 A19:D24 A18:B18 D18 D27" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: standardise Excel export to match import template and restrict student deletion to admin role
</commit_message>
<xml_diff>
--- a/Data_Akun_SkillPassport.xlsx
+++ b/Data_Akun_SkillPassport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Private\Website\skillpas-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE09A76-833F-41B0-A4E1-49D27AABD72E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E67612-C5C6-4D2A-9AB1-136E4ABBC11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="302">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -611,9 +611,6 @@
     <t>walas_hafidz_xii_tkr1</t>
   </si>
   <si>
-    <t>walas_hafidz_xii_tkr3</t>
-  </si>
-  <si>
     <t>M. Teguh Suprihatin, S.Psi</t>
   </si>
   <si>
@@ -936,6 +933,12 @@
   </si>
   <si>
     <t>prod_mesin_02</t>
+  </si>
+  <si>
+    <t>Diana Cholida, S.Pd</t>
+  </si>
+  <si>
+    <t>walas_diana_xii_tkr3</t>
   </si>
 </sst>
 </file>
@@ -1664,13 +1667,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B25" t="s">
         <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D25" s="1">
         <v>123</v>
@@ -2742,13 +2745,13 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>190</v>
+        <v>300</v>
       </c>
       <c r="B102" t="s">
         <v>72</v>
       </c>
       <c r="C102" t="s">
-        <v>192</v>
+        <v>301</v>
       </c>
       <c r="D102" t="s">
         <v>12</v>
@@ -2756,13 +2759,13 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
+        <v>192</v>
+      </c>
+      <c r="B103" t="s">
+        <v>72</v>
+      </c>
+      <c r="C103" t="s">
         <v>193</v>
-      </c>
-      <c r="B103" t="s">
-        <v>72</v>
-      </c>
-      <c r="C103" t="s">
-        <v>194</v>
       </c>
       <c r="D103" t="s">
         <v>12</v>
@@ -2770,13 +2773,13 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B104" t="s">
         <v>72</v>
       </c>
       <c r="C104" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D104" t="s">
         <v>12</v>
@@ -2784,13 +2787,13 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" t="s">
+        <v>72</v>
+      </c>
+      <c r="C105" t="s">
         <v>196</v>
-      </c>
-      <c r="B105" t="s">
-        <v>72</v>
-      </c>
-      <c r="C105" t="s">
-        <v>197</v>
       </c>
       <c r="D105" t="s">
         <v>12</v>
@@ -2798,13 +2801,13 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
+        <v>197</v>
+      </c>
+      <c r="B106" t="s">
+        <v>72</v>
+      </c>
+      <c r="C106" t="s">
         <v>198</v>
-      </c>
-      <c r="B106" t="s">
-        <v>72</v>
-      </c>
-      <c r="C106" t="s">
-        <v>199</v>
       </c>
       <c r="D106" t="s">
         <v>12</v>
@@ -2812,13 +2815,13 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B107" t="s">
         <v>72</v>
       </c>
       <c r="C107" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D107" t="s">
         <v>12</v>
@@ -2826,13 +2829,13 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
+        <v>200</v>
+      </c>
+      <c r="B108" t="s">
+        <v>72</v>
+      </c>
+      <c r="C108" t="s">
         <v>201</v>
-      </c>
-      <c r="B108" t="s">
-        <v>72</v>
-      </c>
-      <c r="C108" t="s">
-        <v>202</v>
       </c>
       <c r="D108" t="s">
         <v>12</v>
@@ -2840,13 +2843,13 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
+        <v>202</v>
+      </c>
+      <c r="B109" t="s">
+        <v>72</v>
+      </c>
+      <c r="C109" t="s">
         <v>203</v>
-      </c>
-      <c r="B109" t="s">
-        <v>72</v>
-      </c>
-      <c r="C109" t="s">
-        <v>204</v>
       </c>
       <c r="D109" t="s">
         <v>12</v>
@@ -2854,13 +2857,13 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
+        <v>204</v>
+      </c>
+      <c r="B110" t="s">
+        <v>72</v>
+      </c>
+      <c r="C110" t="s">
         <v>205</v>
-      </c>
-      <c r="B110" t="s">
-        <v>72</v>
-      </c>
-      <c r="C110" t="s">
-        <v>206</v>
       </c>
       <c r="D110" t="s">
         <v>12</v>
@@ -2868,13 +2871,13 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
+        <v>206</v>
+      </c>
+      <c r="B111" t="s">
+        <v>72</v>
+      </c>
+      <c r="C111" t="s">
         <v>207</v>
-      </c>
-      <c r="B111" t="s">
-        <v>72</v>
-      </c>
-      <c r="C111" t="s">
-        <v>208</v>
       </c>
       <c r="D111" t="s">
         <v>12</v>
@@ -2882,13 +2885,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B112" t="s">
         <v>72</v>
       </c>
       <c r="C112" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D112" t="s">
         <v>12</v>
@@ -2896,13 +2899,13 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
+        <v>209</v>
+      </c>
+      <c r="B113" t="s">
+        <v>72</v>
+      </c>
+      <c r="C113" t="s">
         <v>210</v>
-      </c>
-      <c r="B113" t="s">
-        <v>72</v>
-      </c>
-      <c r="C113" t="s">
-        <v>211</v>
       </c>
       <c r="D113" t="s">
         <v>12</v>
@@ -2910,13 +2913,13 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
+        <v>211</v>
+      </c>
+      <c r="B114" t="s">
+        <v>72</v>
+      </c>
+      <c r="C114" t="s">
         <v>212</v>
-      </c>
-      <c r="B114" t="s">
-        <v>72</v>
-      </c>
-      <c r="C114" t="s">
-        <v>213</v>
       </c>
       <c r="D114" t="s">
         <v>12</v>
@@ -2924,13 +2927,13 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
+        <v>213</v>
+      </c>
+      <c r="B115" t="s">
+        <v>72</v>
+      </c>
+      <c r="C115" t="s">
         <v>214</v>
-      </c>
-      <c r="B115" t="s">
-        <v>72</v>
-      </c>
-      <c r="C115" t="s">
-        <v>215</v>
       </c>
       <c r="D115" t="s">
         <v>12</v>
@@ -2938,13 +2941,13 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
+        <v>215</v>
+      </c>
+      <c r="B116" t="s">
+        <v>72</v>
+      </c>
+      <c r="C116" t="s">
         <v>216</v>
-      </c>
-      <c r="B116" t="s">
-        <v>72</v>
-      </c>
-      <c r="C116" t="s">
-        <v>217</v>
       </c>
       <c r="D116" t="s">
         <v>12</v>
@@ -2952,13 +2955,13 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
+        <v>217</v>
+      </c>
+      <c r="B117" t="s">
+        <v>72</v>
+      </c>
+      <c r="C117" t="s">
         <v>218</v>
-      </c>
-      <c r="B117" t="s">
-        <v>72</v>
-      </c>
-      <c r="C117" t="s">
-        <v>219</v>
       </c>
       <c r="D117" t="s">
         <v>12</v>
@@ -2966,13 +2969,13 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
+        <v>219</v>
+      </c>
+      <c r="B118" t="s">
+        <v>72</v>
+      </c>
+      <c r="C118" t="s">
         <v>220</v>
-      </c>
-      <c r="B118" t="s">
-        <v>72</v>
-      </c>
-      <c r="C118" t="s">
-        <v>221</v>
       </c>
       <c r="D118" t="s">
         <v>12</v>
@@ -2980,13 +2983,13 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
+        <v>221</v>
+      </c>
+      <c r="B119" t="s">
+        <v>72</v>
+      </c>
+      <c r="C119" t="s">
         <v>222</v>
-      </c>
-      <c r="B119" t="s">
-        <v>72</v>
-      </c>
-      <c r="C119" t="s">
-        <v>223</v>
       </c>
       <c r="D119" t="s">
         <v>12</v>
@@ -2994,13 +2997,13 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
+        <v>223</v>
+      </c>
+      <c r="B120" t="s">
+        <v>72</v>
+      </c>
+      <c r="C120" t="s">
         <v>224</v>
-      </c>
-      <c r="B120" t="s">
-        <v>72</v>
-      </c>
-      <c r="C120" t="s">
-        <v>225</v>
       </c>
       <c r="D120" t="s">
         <v>12</v>
@@ -3008,13 +3011,13 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
+        <v>225</v>
+      </c>
+      <c r="B121" t="s">
+        <v>72</v>
+      </c>
+      <c r="C121" t="s">
         <v>226</v>
-      </c>
-      <c r="B121" t="s">
-        <v>72</v>
-      </c>
-      <c r="C121" t="s">
-        <v>227</v>
       </c>
       <c r="D121" t="s">
         <v>12</v>
@@ -3022,13 +3025,13 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
+        <v>227</v>
+      </c>
+      <c r="B122" t="s">
+        <v>72</v>
+      </c>
+      <c r="C122" t="s">
         <v>228</v>
-      </c>
-      <c r="B122" t="s">
-        <v>72</v>
-      </c>
-      <c r="C122" t="s">
-        <v>229</v>
       </c>
       <c r="D122" t="s">
         <v>12</v>
@@ -3036,13 +3039,13 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
+        <v>229</v>
+      </c>
+      <c r="B123" t="s">
+        <v>72</v>
+      </c>
+      <c r="C123" t="s">
         <v>230</v>
-      </c>
-      <c r="B123" t="s">
-        <v>72</v>
-      </c>
-      <c r="C123" t="s">
-        <v>231</v>
       </c>
       <c r="D123" t="s">
         <v>12</v>
@@ -3050,13 +3053,13 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
+        <v>231</v>
+      </c>
+      <c r="B124" t="s">
+        <v>72</v>
+      </c>
+      <c r="C124" t="s">
         <v>232</v>
-      </c>
-      <c r="B124" t="s">
-        <v>72</v>
-      </c>
-      <c r="C124" t="s">
-        <v>233</v>
       </c>
       <c r="D124" t="s">
         <v>12</v>
@@ -3064,13 +3067,13 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
+        <v>233</v>
+      </c>
+      <c r="B125" t="s">
+        <v>72</v>
+      </c>
+      <c r="C125" t="s">
         <v>234</v>
-      </c>
-      <c r="B125" t="s">
-        <v>72</v>
-      </c>
-      <c r="C125" t="s">
-        <v>235</v>
       </c>
       <c r="D125" t="s">
         <v>12</v>
@@ -3084,7 +3087,7 @@
         <v>72</v>
       </c>
       <c r="C126" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D126" t="s">
         <v>12</v>
@@ -3092,13 +3095,13 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
+        <v>236</v>
+      </c>
+      <c r="B127" t="s">
+        <v>72</v>
+      </c>
+      <c r="C127" t="s">
         <v>237</v>
-      </c>
-      <c r="B127" t="s">
-        <v>72</v>
-      </c>
-      <c r="C127" t="s">
-        <v>238</v>
       </c>
       <c r="D127" t="s">
         <v>12</v>
@@ -3106,13 +3109,13 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
+        <v>238</v>
+      </c>
+      <c r="B128" t="s">
+        <v>72</v>
+      </c>
+      <c r="C128" t="s">
         <v>239</v>
-      </c>
-      <c r="B128" t="s">
-        <v>72</v>
-      </c>
-      <c r="C128" t="s">
-        <v>240</v>
       </c>
       <c r="D128" t="s">
         <v>12</v>
@@ -3120,13 +3123,13 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
+        <v>240</v>
+      </c>
+      <c r="B129" t="s">
+        <v>72</v>
+      </c>
+      <c r="C129" t="s">
         <v>241</v>
-      </c>
-      <c r="B129" t="s">
-        <v>72</v>
-      </c>
-      <c r="C129" t="s">
-        <v>242</v>
       </c>
       <c r="D129" t="s">
         <v>12</v>
@@ -3134,13 +3137,13 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B130" t="s">
         <v>72</v>
       </c>
       <c r="C130" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D130" t="s">
         <v>12</v>
@@ -3148,13 +3151,13 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
+        <v>243</v>
+      </c>
+      <c r="B131" t="s">
+        <v>72</v>
+      </c>
+      <c r="C131" t="s">
         <v>244</v>
-      </c>
-      <c r="B131" t="s">
-        <v>72</v>
-      </c>
-      <c r="C131" t="s">
-        <v>245</v>
       </c>
       <c r="D131" t="s">
         <v>12</v>
@@ -3162,13 +3165,13 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
+        <v>245</v>
+      </c>
+      <c r="B132" t="s">
+        <v>72</v>
+      </c>
+      <c r="C132" t="s">
         <v>246</v>
-      </c>
-      <c r="B132" t="s">
-        <v>72</v>
-      </c>
-      <c r="C132" t="s">
-        <v>247</v>
       </c>
       <c r="D132" t="s">
         <v>12</v>
@@ -3176,13 +3179,13 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
+        <v>247</v>
+      </c>
+      <c r="B133" t="s">
+        <v>72</v>
+      </c>
+      <c r="C133" t="s">
         <v>248</v>
-      </c>
-      <c r="B133" t="s">
-        <v>72</v>
-      </c>
-      <c r="C133" t="s">
-        <v>249</v>
       </c>
       <c r="D133" t="s">
         <v>12</v>
@@ -3190,13 +3193,13 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B134" t="s">
         <v>72</v>
       </c>
       <c r="C134" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D134" t="s">
         <v>12</v>
@@ -3204,13 +3207,13 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
+        <v>250</v>
+      </c>
+      <c r="B135" t="s">
+        <v>72</v>
+      </c>
+      <c r="C135" t="s">
         <v>251</v>
-      </c>
-      <c r="B135" t="s">
-        <v>72</v>
-      </c>
-      <c r="C135" t="s">
-        <v>252</v>
       </c>
       <c r="D135" t="s">
         <v>12</v>
@@ -3218,13 +3221,13 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
+        <v>252</v>
+      </c>
+      <c r="B136" t="s">
+        <v>72</v>
+      </c>
+      <c r="C136" t="s">
         <v>253</v>
-      </c>
-      <c r="B136" t="s">
-        <v>72</v>
-      </c>
-      <c r="C136" t="s">
-        <v>254</v>
       </c>
       <c r="D136" t="s">
         <v>12</v>
@@ -3232,13 +3235,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
+        <v>254</v>
+      </c>
+      <c r="B137" t="s">
+        <v>72</v>
+      </c>
+      <c r="C137" t="s">
         <v>255</v>
-      </c>
-      <c r="B137" t="s">
-        <v>72</v>
-      </c>
-      <c r="C137" t="s">
-        <v>256</v>
       </c>
       <c r="D137" t="s">
         <v>12</v>
@@ -3246,13 +3249,13 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B138" t="s">
         <v>72</v>
       </c>
       <c r="C138" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D138" t="s">
         <v>12</v>
@@ -3260,13 +3263,13 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
+        <v>257</v>
+      </c>
+      <c r="B139" t="s">
+        <v>72</v>
+      </c>
+      <c r="C139" t="s">
         <v>258</v>
-      </c>
-      <c r="B139" t="s">
-        <v>72</v>
-      </c>
-      <c r="C139" t="s">
-        <v>259</v>
       </c>
       <c r="D139" t="s">
         <v>12</v>
@@ -3274,13 +3277,13 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
+        <v>259</v>
+      </c>
+      <c r="B140" t="s">
+        <v>72</v>
+      </c>
+      <c r="C140" t="s">
         <v>260</v>
-      </c>
-      <c r="B140" t="s">
-        <v>72</v>
-      </c>
-      <c r="C140" t="s">
-        <v>261</v>
       </c>
       <c r="D140" t="s">
         <v>12</v>
@@ -3288,13 +3291,13 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
+        <v>261</v>
+      </c>
+      <c r="B141" t="s">
+        <v>72</v>
+      </c>
+      <c r="C141" t="s">
         <v>262</v>
-      </c>
-      <c r="B141" t="s">
-        <v>72</v>
-      </c>
-      <c r="C141" t="s">
-        <v>263</v>
       </c>
       <c r="D141" t="s">
         <v>12</v>
@@ -3302,13 +3305,13 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
+        <v>263</v>
+      </c>
+      <c r="B142" t="s">
+        <v>72</v>
+      </c>
+      <c r="C142" t="s">
         <v>264</v>
-      </c>
-      <c r="B142" t="s">
-        <v>72</v>
-      </c>
-      <c r="C142" t="s">
-        <v>265</v>
       </c>
       <c r="D142" t="s">
         <v>12</v>
@@ -3316,13 +3319,13 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B143" t="s">
         <v>72</v>
       </c>
       <c r="C143" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D143" t="s">
         <v>12</v>
@@ -3330,13 +3333,13 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
+        <v>266</v>
+      </c>
+      <c r="B144" t="s">
+        <v>72</v>
+      </c>
+      <c r="C144" t="s">
         <v>267</v>
-      </c>
-      <c r="B144" t="s">
-        <v>72</v>
-      </c>
-      <c r="C144" t="s">
-        <v>268</v>
       </c>
       <c r="D144" t="s">
         <v>12</v>
@@ -3344,13 +3347,13 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
+        <v>268</v>
+      </c>
+      <c r="B145" t="s">
+        <v>72</v>
+      </c>
+      <c r="C145" t="s">
         <v>269</v>
-      </c>
-      <c r="B145" t="s">
-        <v>72</v>
-      </c>
-      <c r="C145" t="s">
-        <v>270</v>
       </c>
       <c r="D145" t="s">
         <v>12</v>
@@ -3358,13 +3361,13 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
+        <v>270</v>
+      </c>
+      <c r="B146" t="s">
+        <v>72</v>
+      </c>
+      <c r="C146" t="s">
         <v>271</v>
-      </c>
-      <c r="B146" t="s">
-        <v>72</v>
-      </c>
-      <c r="C146" t="s">
-        <v>272</v>
       </c>
       <c r="D146" t="s">
         <v>12</v>
@@ -3372,13 +3375,13 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
+        <v>272</v>
+      </c>
+      <c r="B147" t="s">
+        <v>72</v>
+      </c>
+      <c r="C147" t="s">
         <v>273</v>
-      </c>
-      <c r="B147" t="s">
-        <v>72</v>
-      </c>
-      <c r="C147" t="s">
-        <v>274</v>
       </c>
       <c r="D147" t="s">
         <v>12</v>
@@ -3386,13 +3389,13 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
+        <v>274</v>
+      </c>
+      <c r="B148" t="s">
+        <v>72</v>
+      </c>
+      <c r="C148" t="s">
         <v>275</v>
-      </c>
-      <c r="B148" t="s">
-        <v>72</v>
-      </c>
-      <c r="C148" t="s">
-        <v>276</v>
       </c>
       <c r="D148" t="s">
         <v>12</v>
@@ -3400,13 +3403,13 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B149" t="s">
         <v>72</v>
       </c>
       <c r="C149" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D149" t="s">
         <v>12</v>
@@ -3414,13 +3417,13 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
+        <v>277</v>
+      </c>
+      <c r="B150" t="s">
+        <v>72</v>
+      </c>
+      <c r="C150" t="s">
         <v>278</v>
-      </c>
-      <c r="B150" t="s">
-        <v>72</v>
-      </c>
-      <c r="C150" t="s">
-        <v>279</v>
       </c>
       <c r="D150" t="s">
         <v>12</v>
@@ -3428,13 +3431,13 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
+        <v>279</v>
+      </c>
+      <c r="B151" t="s">
+        <v>72</v>
+      </c>
+      <c r="C151" t="s">
         <v>280</v>
-      </c>
-      <c r="B151" t="s">
-        <v>72</v>
-      </c>
-      <c r="C151" t="s">
-        <v>281</v>
       </c>
       <c r="D151" t="s">
         <v>12</v>
@@ -3442,13 +3445,13 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B152" t="s">
         <v>72</v>
       </c>
       <c r="C152" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D152" t="s">
         <v>12</v>
@@ -3456,13 +3459,13 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
+        <v>282</v>
+      </c>
+      <c r="B153" t="s">
+        <v>72</v>
+      </c>
+      <c r="C153" t="s">
         <v>283</v>
-      </c>
-      <c r="B153" t="s">
-        <v>72</v>
-      </c>
-      <c r="C153" t="s">
-        <v>284</v>
       </c>
       <c r="D153" t="s">
         <v>12</v>
@@ -3470,13 +3473,13 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
+        <v>284</v>
+      </c>
+      <c r="B154" t="s">
+        <v>72</v>
+      </c>
+      <c r="C154" t="s">
         <v>285</v>
-      </c>
-      <c r="B154" t="s">
-        <v>72</v>
-      </c>
-      <c r="C154" t="s">
-        <v>286</v>
       </c>
       <c r="D154" t="s">
         <v>12</v>
@@ -3484,13 +3487,13 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B155" t="s">
         <v>72</v>
       </c>
       <c r="C155" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D155" t="s">
         <v>12</v>
@@ -3498,13 +3501,13 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
+        <v>287</v>
+      </c>
+      <c r="B156" t="s">
+        <v>72</v>
+      </c>
+      <c r="C156" t="s">
         <v>288</v>
-      </c>
-      <c r="B156" t="s">
-        <v>72</v>
-      </c>
-      <c r="C156" t="s">
-        <v>289</v>
       </c>
       <c r="D156" t="s">
         <v>12</v>
@@ -3512,13 +3515,13 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
+        <v>289</v>
+      </c>
+      <c r="B157" t="s">
+        <v>72</v>
+      </c>
+      <c r="C157" t="s">
         <v>290</v>
-      </c>
-      <c r="B157" t="s">
-        <v>72</v>
-      </c>
-      <c r="C157" t="s">
-        <v>291</v>
       </c>
       <c r="D157" t="s">
         <v>12</v>
@@ -3526,13 +3529,13 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B158" t="s">
         <v>72</v>
       </c>
       <c r="C158" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D158" t="s">
         <v>12</v>
@@ -3540,13 +3543,13 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
+        <v>292</v>
+      </c>
+      <c r="B159" t="s">
+        <v>72</v>
+      </c>
+      <c r="C159" t="s">
         <v>293</v>
-      </c>
-      <c r="B159" t="s">
-        <v>72</v>
-      </c>
-      <c r="C159" t="s">
-        <v>294</v>
       </c>
       <c r="D159" t="s">
         <v>12</v>
@@ -3554,13 +3557,13 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
+        <v>294</v>
+      </c>
+      <c r="B160" t="s">
+        <v>72</v>
+      </c>
+      <c r="C160" t="s">
         <v>295</v>
-      </c>
-      <c r="B160" t="s">
-        <v>72</v>
-      </c>
-      <c r="C160" t="s">
-        <v>296</v>
       </c>
       <c r="D160" t="s">
         <v>12</v>
@@ -3568,13 +3571,13 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
+        <v>296</v>
+      </c>
+      <c r="B161" t="s">
+        <v>72</v>
+      </c>
+      <c r="C161" t="s">
         <v>297</v>
-      </c>
-      <c r="B161" t="s">
-        <v>72</v>
-      </c>
-      <c r="C161" t="s">
-        <v>298</v>
       </c>
       <c r="D161" t="s">
         <v>12</v>
@@ -3584,7 +3587,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D17 A27:B27 A26:B26 D26 A29:D161 A28:B28 D28 A19:D24 A18:B18 D18 D27" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D17 A27:B27 A26:B26 D26 A29:D101 A28:B28 D28 A19:D24 A18:B18 D18 D27 A103:D161 B102 D102" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>